<commit_message>
Update Playa Dorada ranking with 18 keywords and domain sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ued7r3VpTHoLV9PJaTphTG
</commit_message>
<xml_diff>
--- a/ranking-playadorada.xlsx
+++ b/ranking-playadorada.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Ranking" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dominios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,14 +444,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -492,20 +493,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>playa dorada panama</t>
+          <t>playa dorada panamá</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>/en/home/ (también /en/location/ 7, /amenities 8)</t>
+          <t>/en/home/ (/location 6, /news live 7, /amenities 8, /discover 9)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Facebook, glp.com.pa, Instagram, Panama Relocation Tours, InmoPanama</t>
+          <t>Facebook, glp.com.pa, Panama Relocation Tours, InmoPanama</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -520,20 +521,20 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>playa dorada vacamonte</t>
+          <t>playa dorada panama</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>/blog/noticias-es/venta-casas-vacamonte/</t>
+          <t>/en/home/ (/location 7, /amenities 8)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>glp.com.pa, TikTok, SkyscraperCity, Compreoalquile, Mitula</t>
+          <t>Facebook, glp.com.pa, Instagram, Panama Relocation Tours, InmoPanama</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -548,22 +549,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>playa dorada arraijan</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>8 y 9</t>
-        </is>
+          <t>playa dorada panamá ubicación</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nota 'Una experiencia para vivir y repetir en Arraiján' (EN y ES)</t>
+          <t>/en/location/ (/home 7, blog propiedad-asequible 8, /connectivity 9)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Booking, Facebook, Panama Relocation Tours, InmoPanama</t>
+          <t>Caja de Ahorros, Facebook, glp.com.pa, Relocation Tours, Mapcarta</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -578,20 +577,20 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>playa dorada residences</t>
+          <t>playa dorada panama rentals</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>/en/home/</t>
+          <t>/en/rentals/ (home 9)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Vrbo, Tripadvisor, otros Playa Dorada (RD, Italia)</t>
+          <t>Encuentra24 (x2), glp.com.pa, Tripadvisor, Panamawise, InmoPanama</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -606,7 +605,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>playa dorada panama rentals</t>
+          <t>donde queda playa dorada en panama</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -614,12 +613,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>/en/rentals/</t>
+          <t>/en/location/ (home 8, amenities 9, connectivity 10)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Encuentra24 (x2), glp.com.pa, Panamawise</t>
+          <t>Facebook, glp.com.pa, Relocation Tours, Grupo GEA, Parque Logístico, Mapcarta</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -634,20 +633,20 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>donde queda playa dorada en panama</t>
+          <t>playa dorada vacamonte</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>/en/location/</t>
+          <t>/blog/noticias-es/venta-casas-vacamonte/</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Facebook, glp.com.pa, Panama Relocation Tours, Grupo GEA</t>
+          <t>glp.com.pa, TikTok, SkyscraperCity, Compreoalquile, Mitula, Parque Logístico, InmoPanama</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -662,20 +661,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>playa dorada casas</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>8</v>
+          <t>playa dorada arraijan</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>8 y 9</t>
+        </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>/casas/</t>
+          <t>Nota 'Una experiencia para vivir y repetir en Arraiján' (EN y ES)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Idealista (Lanzarote), Encuentra24, glp.com.pa</t>
+          <t>Booking (x2), Facebook (x2), Relocation Tours, Travelmyth, InmoPanama</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -690,7 +691,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>playa dorada panama oeste</t>
+          <t>playa dorada residences</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -698,12 +699,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>/en/home/ (/amenities 9, /location 10)</t>
+          <t>/en/home/ (news live 9)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Facebook, Relocation Tours, Instagram, glp.com.pa, Ribera</t>
+          <t>Vrbo, Tripadvisor, Xanadu (RD), playadoradaresidence.com, rentbyowner, playadorada.eu</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -718,20 +719,20 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>bay club playa dorada</t>
+          <t>playa dorada casas</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>/club-de-playa/</t>
+          <t>/casas/</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Instagram, bayclubpanama.com</t>
+          <t>Idealista (x2), Encuentra24, glp.com.pa, propiedades.com, Lamudi, InmoPanama</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -746,27 +747,25 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>playa dorada panama real estate</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>No top 9</t>
-        </is>
+          <t>playa dorada panama oeste</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>/en/home/ (amenities 9, location 10)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Encuentra24, Casa Solution, glp.com.pa, Panamawise</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Sin ranking</t>
+          <t>Facebook (x1), Relocation Tours, Instagram, glp.com.pa, Ribera, Mapcarta, Ocean Front</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>En top 10</t>
         </is>
       </c>
     </row>
@@ -776,27 +775,25 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>alquiler en playa dorada</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>No aparece</t>
-        </is>
+          <t>playa dorada panama rentals long term</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>/en/news/beach-houses-in-panama... (/en/rentals/ 10)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Vrbo, Booking, Playas Doradas (Argentina)</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Sin ranking</t>
+          <t>glp.com.pa, Encuentra24 (x3), Tripadvisor, Viviun, Relocation Tours</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>En top 10</t>
         </is>
       </c>
     </row>
@@ -806,25 +803,201 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>bay club playa dorada</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>/club-de-playa/</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Instagram, Infinitum, Puerto Plata, Rantan, bayclubpanama.com, Playa Dorada Golf, Blue Bay, Facebook</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>En top 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>playa dorado panama</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>/en/location/</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Facebook (x2), glp.com.pa, Wikipedia, Relocation Tours, Instagram, Grupo GEA, bayclubpanama.com, InmoPanama</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>En top 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>playa dorada panama real estate</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>No aparece (top 9)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Encuentra24, Casa Solution, glp.com.pa, Panamawise, New World RE, InmoPanama</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Sin ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>alquiler en playa dorada</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>No aparece (top 9)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Vrbo, Booking, Playas Doradas (Argentina), InmoPanama</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Sin ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>apartamentos en playa dorada</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>No aparece (top 9)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Trivago (RD), Plusval (RD), Encuentra24, Vrbo, Vetas</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Sin ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
           <t>playa dorada</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>No aparece</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>No aparece (top 9)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Playa Dorada, Puerto Plata (República Dominicana)</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Tripadvisor, Expedia, Playa Dorada Puerto Plata (RD)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Sin ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>playa dorado</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>No aparece (top 9)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Apple Maps (Dorado, PR), Instagram, Tripadvisor (RD)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Sin ranking</t>
         </is>
@@ -836,6 +1009,162 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dominio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Keywords donde aparece (de 18)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>playadorada.com.pa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sitio oficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>glp.com.pa</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Desarrollador</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram Playa Dorada</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Redes oficiales</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>inmopanama.com</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Portal inmobiliario</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>panamarelocationtours.com</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Contenido expats</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Encuentra24</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Portal venta/alquiler</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mapcarta.com</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Booking/Vrbo/Tripadvisor</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Alquiler vacacional</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -850,14 +1179,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Posiciones aproximadas: orden de resultados de búsqueda web (EE. UU.), no datos de Google Search Console.</t>
+          <t>Posiciones aproximadas: orden de resultados de búsqueda web (EE. UU., 9-10 resultados), no Google Panamá ni GSC.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Para posiciones exactas, exportar GSC &gt; Rendimiento &gt; Consultas &gt; Posición media.</t>
+          <t>Para posiciones reales: GSC &gt; Rendimiento &gt; Consultas &gt; filtro País: Panamá.</t>
         </is>
       </c>
     </row>

</xml_diff>